<commit_message>
UI: Coloca etiquetas directamente sobre los puntos y elimina leyenda redundante en Panel A
</commit_message>
<xml_diff>
--- a/Datos/Tabla1.xlsx
+++ b/Datos/Tabla1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Laboratorio de Ambientes Inteligentes\Proyecto Inundaciones\Proyecto_Recomendaciones_Inundaciones\Datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFB9DFC6-A6C1-4598-B9F4-374E1A2D3678}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CA38F24-1C96-4C29-9298-1BB6F96C2632}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{D3AFEBD6-96F4-4E36-97A2-D1F1D80A7D7C}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="104">
   <si>
     <t>Municipio</t>
   </si>
@@ -336,6 +336,21 @@
   </si>
   <si>
     <t>0.2323481341377387</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>II</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t>III</t>
+  </si>
+  <si>
+    <t>IV</t>
   </si>
 </sst>
 </file>
@@ -401,7 +416,10 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="11">
+  <dxfs count="12">
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -465,21 +483,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4BA8149E-779E-475F-A60C-3438B14A5984}" name="Tabla1" displayName="Tabla1" ref="A1:I13" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
-  <autoFilter ref="A1:I13" xr:uid="{4BA8149E-779E-475F-A60C-3438B14A5984}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4BA8149E-779E-475F-A60C-3438B14A5984}" name="Tabla1" displayName="Tabla1" ref="A1:J13" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
+  <autoFilter ref="A1:J13" xr:uid="{4BA8149E-779E-475F-A60C-3438B14A5984}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I13">
     <sortCondition ref="A1:A13"/>
   </sortState>
-  <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{39D106A7-194E-46E5-8605-4ED96635F332}" name="Municipio" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{57551B40-141C-46B9-9D9D-2F7A24A200C8}" name="IVS" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{C30EEC64-C227-45FB-9F98-F4F5CEF104BE}" name="DIM_SS" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{4D6F3DDB-69ED-4AF8-B4A4-84641CFB14CD}" name="DIM_EF" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{79C057E6-C218-44B0-8D73-3A00881DA5A8}" name="DIM_CA" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{B87DB94D-CC00-4E94-90A2-7CB24B0D6A62}" name="DIM_GV" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{5BB92E3D-5CDD-4C9B-A074-933413109150}" name="ICI_Gen" dataDxfId="2"/>
-    <tableColumn id="8" xr3:uid="{40327DFA-6B4E-4081-BBD4-4385F5123D7D}" name="ICI_Rsg" dataDxfId="1"/>
-    <tableColumn id="9" xr3:uid="{789913F7-CC80-4792-905A-7F9DA0C3FD7D}" name="ICI_Comp" dataDxfId="0"/>
+  <tableColumns count="10">
+    <tableColumn id="1" xr3:uid="{39D106A7-194E-46E5-8605-4ED96635F332}" name="Municipio" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{57551B40-141C-46B9-9D9D-2F7A24A200C8}" name="IVS" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{C30EEC64-C227-45FB-9F98-F4F5CEF104BE}" name="DIM_SS" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{4D6F3DDB-69ED-4AF8-B4A4-84641CFB14CD}" name="DIM_EF" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{79C057E6-C218-44B0-8D73-3A00881DA5A8}" name="DIM_CA" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{B87DB94D-CC00-4E94-90A2-7CB24B0D6A62}" name="DIM_GV" dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{5BB92E3D-5CDD-4C9B-A074-933413109150}" name="ICI_Gen" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{40327DFA-6B4E-4081-BBD4-4385F5123D7D}" name="ICI_Rsg" dataDxfId="2"/>
+    <tableColumn id="9" xr3:uid="{789913F7-CC80-4792-905A-7F9DA0C3FD7D}" name="ICI_Comp" dataDxfId="1"/>
+    <tableColumn id="10" xr3:uid="{7DD18844-935A-49AE-B047-6FD9BEDE0E9C}" name="C" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -782,14 +801,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28EBBEA0-3CDE-4526-9D14-D2CFDC34215C}">
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="11.08984375" customWidth="1"/>
     <col min="9" max="9" width="15.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -817,8 +836,11 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J1" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
@@ -846,8 +868,11 @@
       <c r="I2" s="4" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J2" s="2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>14</v>
       </c>
@@ -875,8 +900,11 @@
       <c r="I3" s="4" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J3" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -904,8 +932,11 @@
       <c r="I4" s="4" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J4" s="2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
@@ -933,8 +964,11 @@
       <c r="I5" s="4" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J5" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -962,8 +996,11 @@
       <c r="I6" s="4" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J6" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
@@ -991,8 +1028,11 @@
       <c r="I7" s="4" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J7" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>17</v>
       </c>
@@ -1020,8 +1060,11 @@
       <c r="I8" s="4" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="J8" s="2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>12</v>
       </c>
@@ -1049,8 +1092,11 @@
       <c r="I9" s="4" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J9" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>11</v>
       </c>
@@ -1078,8 +1124,11 @@
       <c r="I10" s="4" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J10" s="2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>18</v>
       </c>
@@ -1107,8 +1156,11 @@
       <c r="I11" s="4" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J11" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>16</v>
       </c>
@@ -1136,8 +1188,11 @@
       <c r="I12" s="4" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J12" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>15</v>
       </c>
@@ -1165,8 +1220,11 @@
       <c r="I13" s="4" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J13" s="2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B16" s="3"/>
     </row>
   </sheetData>

</xml_diff>